<commit_message>
Improve flowchart edge routing
</commit_message>
<xml_diff>
--- a/examples/purchase_process.xlsx
+++ b/examples/purchase_process.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="フロー図" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="注記" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="フロー図" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注記" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'フロー図'!$A$1:$Q$8</definedName>
@@ -209,6 +209,1314 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="Edge_22"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2228850" y="1682750"/>
+          <a:ext cx="342900" cy="114300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="50000"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="83333" y="50000"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Edge_23"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3695700" y="1682750"/>
+          <a:ext cx="1809750" cy="2400300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="3157" y="2380"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="2380"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="97619"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="96842" y="97619"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="Edge_25"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3695700" y="1682750"/>
+          <a:ext cx="342900" cy="1257300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="4545"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="4545"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="95454"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="95454"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="Edge_27"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5162550" y="2825750"/>
+          <a:ext cx="342900" cy="1257300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="4545"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="4545"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="95454"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="95454"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="29" name="Edge_29"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5162550" y="1682750"/>
+          <a:ext cx="342900" cy="1257300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="95454"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="95454"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="4545"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="4545"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1409700</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1019175</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="Edge_31"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1609725" y="1682750"/>
+          <a:ext cx="5133975" cy="504825"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="98886" y="11320"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="98886" y="88679"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1113" y="88679"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1113" y="54716"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="32" name="Edge_32"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6629400" y="3968750"/>
+          <a:ext cx="342900" cy="114300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="50000"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="83333" y="50000"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="33" name="Edge_33"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8096250" y="3968750"/>
+          <a:ext cx="342900" cy="114300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="50000"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="83333" y="50000"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="34" name="Edge_34"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9563100" y="3683000"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="85714"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="14285"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>914400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="36" name="Edge_36"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9563100" y="3968750"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="14285"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="85714"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>733425</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1409700</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>1085850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="Edge_38"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7477125" y="4187825"/>
+          <a:ext cx="3667125" cy="352425"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="98441" y="35135"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="98441" y="83783"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1558" y="83783"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1558" y="16216"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="39" name="Edge_39"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11029950" y="3683000"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="14285"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="85714"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="Edge_40"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12496800" y="3968750"/>
+          <a:ext cx="342900" cy="1257300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="4545"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="4545"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="95454"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="95454"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="Edge_41"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13963650" y="5111750"/>
+          <a:ext cx="342900" cy="114300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="50000"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="83333" y="50000"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="42" name="Edge_42"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15430500" y="4826000"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="85714"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="14285"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>914400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="Edge_44"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15430500" y="5111750"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="14285"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="85714"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>733425</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>790575</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>695325</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="46" name="Edge_46"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11877675" y="4187825"/>
+          <a:ext cx="4514850" cy="1104900"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="98734" y="94827"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="98734" y="50000"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1265" y="50000"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="1265" y="5172"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="47" name="Edge_47"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16897350" y="4826000"/>
+          <a:ext cx="342900" cy="1543050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="3703"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="3703"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="96296"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="96296"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="48" name="Edge_48"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18364200" y="6254750"/>
+          <a:ext cx="342900" cy="114300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="50000"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="83333" y="50000"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="49" name="Edge_49"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19831050" y="5969000"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="85714"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="14285"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>914400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="51" name="Edge_51"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19831050" y="6254750"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="14285"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="85714"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>733425</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>1409700</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1085850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="Edge_53"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19211925" y="6473825"/>
+          <a:ext cx="2200275" cy="352425"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="97402" y="35135"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="97402" y="83783"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="2597" y="83783"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="2597" y="16216"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="54" name="Edge_54"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21297900" y="5969000"/>
+          <a:ext cx="342900" cy="400050"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="14285"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="50000" y="14285"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="50000" y="85714"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="83333" y="85714"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>628650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="55" name="Edge_55"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22764750" y="6254750"/>
+          <a:ext cx="342900" cy="114300"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="100000" b="100000"/>
+          <a:pathLst>
+            <a:path w="100000" h="100000">
+              <a:moveTo>
+                <a:pt x="16666" y="50000"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="83333" y="50000"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="333333"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>352425</xdr:rowOff>
@@ -1268,93 +2576,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>571501</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="22" name="Edge_22"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="2" idx="3"/>
-          <a:endCxn id="3" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2286000" y="1739900"/>
-          <a:ext cx="228600" cy="1"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="23" name="Edge_23"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="3" idx="3"/>
-          <a:endCxn id="6" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3752850" y="1739900"/>
-          <a:ext cx="1695450" cy="2286000"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>1057275</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1364,7 +2594,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3848100" y="2225675"/>
+          <a:off x="3848100" y="3368675"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1398,54 +2628,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="25" name="Edge_25"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="3" idx="3"/>
-          <a:endCxn id="4" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3752850" y="1739900"/>
-          <a:ext cx="228600" cy="1143000"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1447800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>771525</xdr:rowOff>
+      <xdr:rowOff>200025</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>942975</xdr:rowOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1454,7 +2645,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3848100" y="1939925"/>
+          <a:off x="3848100" y="2511425"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1488,54 +2679,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="27" name="Edge_27"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="4" idx="3"/>
-          <a:endCxn id="6" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5219700" y="2882900"/>
-          <a:ext cx="228600" cy="1143000"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1447800</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>771525</xdr:rowOff>
+      <xdr:rowOff>200025</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>942975</xdr:rowOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1544,7 +2696,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5314950" y="3082925"/>
+          <a:off x="5314950" y="3654425"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1578,54 +2730,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
+      <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="29" name="Edge_29"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="4" idx="3"/>
-          <a:endCxn id="5" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="5219700" y="1739900"/>
-          <a:ext cx="228600" cy="1143000"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1447800</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>200025</xdr:rowOff>
+      <xdr:rowOff>771525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>371475</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>942975</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1634,7 +2747,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5314950" y="2511425"/>
+          <a:off x="5314950" y="1939925"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1667,192 +2780,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>203200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>352425</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="31" name="Back_31"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="5" idx="0"/>
-          <a:endCxn id="2" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1666875" y="965200"/>
-          <a:ext cx="4400550" cy="555625"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="100000" b="100000"/>
-          <a:pathLst>
-            <a:path w="100000" h="100000">
-              <a:moveTo>
-                <a:pt x="100000" y="100000"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="100000" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="100000"/>
-              </a:lnTo>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571501</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="32" name="Edge_32"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="6" idx="3"/>
-          <a:endCxn id="7" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6686550" y="4025900"/>
-          <a:ext cx="228600" cy="1"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571501</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="33" name="Edge_33"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="7" idx="3"/>
-          <a:endCxn id="8" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8153400" y="4025900"/>
-          <a:ext cx="228600" cy="1"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="34" name="Edge_34"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="8" idx="3"/>
-          <a:endCxn id="10" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="9620250" y="3740150"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>414337</xdr:rowOff>
+      <xdr:rowOff>271462</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>585787</xdr:rowOff>
+      <xdr:rowOff>442912</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1861,7 +2798,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9715500" y="3868737"/>
+          <a:off x="9715500" y="3725862"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1895,54 +2832,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>857250</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="36" name="Edge_36"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="8" idx="3"/>
-          <a:endCxn id="9" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9620250" y="4025900"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>557212</xdr:rowOff>
+      <xdr:rowOff>700087</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>728662</xdr:rowOff>
+      <xdr:rowOff>871537</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1951,7 +2849,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9715500" y="4011612"/>
+          <a:off x="9715500" y="4154487"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1984,231 +2882,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>203200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>638175</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="38" name="Back_38"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="9" idx="0"/>
-          <a:endCxn id="7" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7534275" y="965200"/>
-          <a:ext cx="2933700" cy="3127375"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="100000" b="100000"/>
-          <a:pathLst>
-            <a:path w="100000" h="100000">
-              <a:moveTo>
-                <a:pt x="100000" y="100000"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="100000" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="90862"/>
-              </a:lnTo>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="39" name="Edge_39"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="10" idx="3"/>
-          <a:endCxn id="11" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11087100" y="3740150"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="40" name="Edge_40"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="11" idx="3"/>
-          <a:endCxn id="12" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="12553950" y="4025900"/>
-          <a:ext cx="228600" cy="1143000"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>571501</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="41" name="Edge_41"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="12" idx="3"/>
-          <a:endCxn id="13" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14020800" y="5168900"/>
-          <a:ext cx="228600" cy="1"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="42" name="Edge_42"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="13" idx="3"/>
-          <a:endCxn id="15" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="15487650" y="4883150"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>414337</xdr:rowOff>
+      <xdr:rowOff>271462</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>585787</xdr:rowOff>
+      <xdr:rowOff>442912</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2217,7 +2900,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15582900" y="5011737"/>
+          <a:off x="15582900" y="4868862"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2251,54 +2934,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>857250</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="44" name="Edge_44"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="13" idx="3"/>
-          <a:endCxn id="14" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15487650" y="5168900"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>557212</xdr:rowOff>
+      <xdr:rowOff>700087</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>728662</xdr:rowOff>
+      <xdr:rowOff>871537</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2307,7 +2951,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15582900" y="5154612"/>
+          <a:off x="15582900" y="5297487"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2340,192 +2984,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>203200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>638175</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="46" name="Back_46"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="14" idx="0"/>
-          <a:endCxn id="11" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11934825" y="965200"/>
-          <a:ext cx="4400550" cy="4270375"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="100000" b="100000"/>
-          <a:pathLst>
-            <a:path w="100000" h="100000">
-              <a:moveTo>
-                <a:pt x="100000" y="100000"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="100000" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="66542"/>
-              </a:lnTo>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="47" name="Edge_47"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="15" idx="3"/>
-          <a:endCxn id="16" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="16954500" y="4883150"/>
-          <a:ext cx="228600" cy="1428750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571501</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="48" name="Edge_48"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="16" idx="3"/>
-          <a:endCxn id="17" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18421350" y="6311900"/>
-          <a:ext cx="228600" cy="1"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="49" name="Edge_49"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="17" idx="3"/>
-          <a:endCxn id="19" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="19888200" y="6026150"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>414337</xdr:rowOff>
+      <xdr:rowOff>271462</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>585787</xdr:rowOff>
+      <xdr:rowOff>442912</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2534,7 +3002,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19983450" y="6154737"/>
+          <a:off x="19983450" y="6011862"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2568,54 +3036,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>857250</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="51" name="Edge_51"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="17" idx="3"/>
-          <a:endCxn id="18" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19888200" y="6311900"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>13</xdr:col>
       <xdr:colOff>1447800</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>557212</xdr:rowOff>
+      <xdr:rowOff>700087</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>728662</xdr:rowOff>
+      <xdr:rowOff>871537</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2624,7 +3053,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19983450" y="6297612"/>
+          <a:off x="19983450" y="6440487"/>
           <a:ext cx="476250" cy="171450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2653,143 +3082,6 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>203200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>638175</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="53" name="Back_53"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="18" idx="0"/>
-          <a:endCxn id="17" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19269075" y="965200"/>
-          <a:ext cx="1466850" cy="5413375"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="100000" b="100000"/>
-          <a:pathLst>
-            <a:path w="100000" h="100000">
-              <a:moveTo>
-                <a:pt x="100000" y="100000"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="100000" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="0"/>
-              </a:lnTo>
-              <a:lnTo>
-                <a:pt x="0" y="94721"/>
-              </a:lnTo>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="54" name="Edge_54"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="19" idx="3"/>
-          <a:endCxn id="20" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="21355050" y="6026150"/>
-          <a:ext cx="228600" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1352550</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>571501</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="55" name="Edge_55"/>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="20" idx="3"/>
-          <a:endCxn id="21" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="22821900" y="6311900"/>
-          <a:ext cx="228600" cy="1"/>
-        </a:xfrm>
-        <a:prstGeom prst="bentConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="333333"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>